<commit_message>
Changes to make teaching data file more human manageable.
</commit_message>
<xml_diff>
--- a/src/make_cv/files/Teaching/teaching evaluation data.xlsx
+++ b/src/make_cv/files/Teaching/teaching evaluation data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bhelenbr/Codes/make_cv/src/make_cv/files/Teaching/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22CA3A21-3FAF-2340-831F-D10C52700CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B9A8DD-D5E9-BD4A-8340-E9FC06FB76CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4440" yWindow="760" windowWidth="39160" windowHeight="18280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$AC$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$F$41</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>STRM</t>
   </si>
@@ -31,82 +31,28 @@
     <t>term</t>
   </si>
   <si>
-    <t>school</t>
-  </si>
-  <si>
-    <t>course</t>
-  </si>
-  <si>
-    <t>course_num</t>
-  </si>
-  <si>
-    <t>course_section</t>
-  </si>
-  <si>
     <t>course_title</t>
   </si>
   <si>
-    <t>INSTR_NA</t>
-  </si>
-  <si>
-    <t>count_evals</t>
-  </si>
-  <si>
     <t>enrollment</t>
   </si>
   <si>
-    <t>Particip</t>
-  </si>
-  <si>
-    <t>question</t>
-  </si>
-  <si>
-    <t>a1</t>
-  </si>
-  <si>
-    <t>a1_pct</t>
-  </si>
-  <si>
-    <t>a2</t>
-  </si>
-  <si>
-    <t>a2_pct</t>
-  </si>
-  <si>
-    <t>a3</t>
-  </si>
-  <si>
-    <t>a3_pct</t>
-  </si>
-  <si>
-    <t>a4</t>
-  </si>
-  <si>
-    <t>a4_pct</t>
-  </si>
-  <si>
-    <t>a5</t>
-  </si>
-  <si>
-    <t>a5_pct</t>
-  </si>
-  <si>
-    <t>na</t>
-  </si>
-  <si>
-    <t>na_pct</t>
-  </si>
-  <si>
-    <t>Calculated Mean</t>
-  </si>
-  <si>
-    <t>Question</t>
-  </si>
-  <si>
-    <t>Weighted Average</t>
-  </si>
-  <si>
     <t>combined_course_num</t>
+  </si>
+  <si>
+    <t>combined_num_sec</t>
+  </si>
+  <si>
+    <t>count_19</t>
+  </si>
+  <si>
+    <t>mean_19</t>
+  </si>
+  <si>
+    <t>count_20</t>
+  </si>
+  <si>
+    <t>mean_20</t>
   </si>
 </sst>
 </file>
@@ -470,10 +416,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.5" customWidth="1"/>
+    <col min="4" max="4" width="23.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -481,16 +435,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -504,64 +458,10 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC41" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC41">
+  <autoFilter ref="A1:F41" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F41">
       <sortCondition ref="B1:B41"/>
     </sortState>
   </autoFilter>

</xml_diff>

<commit_message>
Changes to update teaching output
</commit_message>
<xml_diff>
--- a/src/make_cv/files/Teaching/teaching evaluation data.xlsx
+++ b/src/make_cv/files/Teaching/teaching evaluation data.xlsx
@@ -1,33 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bhelenbr/Codes/make_cv/src/make_cv/files/Teaching/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{703A6433-6631-E04B-8732-A8A5F03CA954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F73D28A-F8A1-8E4A-93EB-055E4DA7F752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="2" r:id="rId1"/>
     <sheet name="Data" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Data!$A$1:$F$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Data!$A$1:$E$41</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
-  <si>
-    <t>STRM</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
   <si>
     <t>term</t>
   </si>
@@ -62,9 +59,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>integer used to chronologically sort terms.  I use this formula: (year-2019)*10 +X where X is 2 for spring, 4 for summer, and 6 for fall.</t>
-  </si>
-  <si>
     <t>text description of term i.e. Fall 20222</t>
   </si>
   <si>
@@ -102,6 +96,15 @@
   </si>
   <si>
     <t>Finite Element Methods</t>
+  </si>
+  <si>
+    <t>ME585-02/CE538-02</t>
+  </si>
+  <si>
+    <t>component</t>
+  </si>
+  <si>
+    <t>optional - include if you have classes with separate "LAB", "LEC", "DIS", or "TUT" components</t>
   </si>
 </sst>
 </file>
@@ -465,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{507FBD4F-34E0-9946-B1F4-8507B94D1541}">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.5" customWidth="1"/>
@@ -474,98 +477,98 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>6</v>
@@ -576,40 +579,63 @@
       <c r="I14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15">
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15">
+        <v>20</v>
+      </c>
+      <c r="F15">
+        <v>16</v>
+      </c>
+      <c r="G15">
+        <v>4.53</v>
+      </c>
+      <c r="H15">
+        <v>16</v>
+      </c>
+      <c r="I15">
+        <v>4.79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16">
         <v>12</v>
       </c>
-      <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15">
-        <v>20</v>
-      </c>
-      <c r="G15">
-        <v>16</v>
-      </c>
-      <c r="H15">
-        <v>4.53</v>
-      </c>
-      <c r="I15">
-        <v>16</v>
-      </c>
-      <c r="J15">
-        <v>4.79</v>
+      <c r="F16">
+        <v>8</v>
+      </c>
+      <c r="G16">
+        <v>3.9</v>
+      </c>
+      <c r="H16">
+        <v>8</v>
+      </c>
+      <c r="I16">
+        <v>4.0999999999999996</v>
       </c>
     </row>
   </sheetData>
@@ -619,35 +645,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.5" customWidth="1"/>
-    <col min="4" max="4" width="23.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.5" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -658,14 +683,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F41" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F41">
-      <sortCondition ref="B1:B41"/>
+  <autoFilter ref="A1:E41" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E41">
+      <sortCondition ref="A1:A41"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>